<commit_message>
breakpoints + desc evol tempo itemsets
</commit_message>
<xml_diff>
--- a/eucast_breakpoints/breakpoints_recap.xlsx
+++ b/eucast_breakpoints/breakpoints_recap.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hodbere\Documents\GitHub\exploring_MDR_patterns\eucast_breakpoints\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hodbert-e\Documents\GitHub\exploring_MDR_patterns\eucast_breakpoints\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DBA5B9E-E1D3-4D6A-922A-ECFBA2FA3962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA63B542-05D3-4A17-A541-24BB16060983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-75" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="brut" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1260" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="968" uniqueCount="110">
   <si>
     <t>Class</t>
   </si>
@@ -350,6 +350,12 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>2020 to 2022 MIC breakpoint (mg/L)</t>
+  </si>
+  <si>
+    <t>2020 to 2022 Zone diameter breakpoint (mm)</t>
   </si>
 </sst>
 </file>
@@ -660,10 +666,40 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -678,32 +714,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -712,27 +738,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1039,46 +1045,46 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="E1" s="12"/>
-      <c r="F1" s="11" t="s">
+      <c r="E1" s="27"/>
+      <c r="F1" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="G1" s="12"/>
-      <c r="H1" s="11" t="s">
+      <c r="G1" s="27"/>
+      <c r="H1" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="I1" s="12"/>
-      <c r="J1" s="11" t="s">
+      <c r="I1" s="27"/>
+      <c r="J1" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="K1" s="12"/>
-      <c r="L1" s="11" t="s">
+      <c r="K1" s="27"/>
+      <c r="L1" s="26" t="s">
         <v>94</v>
       </c>
-      <c r="M1" s="12"/>
-      <c r="N1" s="11" t="s">
+      <c r="M1" s="27"/>
+      <c r="N1" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="O1" s="12"/>
-      <c r="P1" s="11" t="s">
+      <c r="O1" s="27"/>
+      <c r="P1" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="Q1" s="12"/>
-      <c r="R1" s="11" t="s">
+      <c r="Q1" s="27"/>
+      <c r="R1" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="S1" s="12"/>
-      <c r="T1" s="11" t="s">
+      <c r="S1" s="27"/>
+      <c r="T1" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="U1" s="12"/>
-      <c r="V1" s="11" t="s">
+      <c r="U1" s="27"/>
+      <c r="V1" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="W1" s="17"/>
+      <c r="W1" s="28"/>
     </row>
     <row r="2" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6"/>
@@ -1146,7 +1152,7 @@
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="29" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
@@ -1217,7 +1223,7 @@
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A4" s="14"/>
+      <c r="A4" s="30"/>
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
@@ -1286,7 +1292,7 @@
       </c>
     </row>
     <row r="5" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="15"/>
+      <c r="A5" s="31"/>
       <c r="B5" s="4" t="s">
         <v>8</v>
       </c>
@@ -1426,7 +1432,7 @@
       </c>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="29" t="s">
         <v>13</v>
       </c>
       <c r="B7" s="3" t="s">
@@ -1497,7 +1503,7 @@
       </c>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A8" s="14"/>
+      <c r="A8" s="30"/>
       <c r="B8" s="3" t="s">
         <v>16</v>
       </c>
@@ -1566,7 +1572,7 @@
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A9" s="14"/>
+      <c r="A9" s="30"/>
       <c r="B9" s="3" t="s">
         <v>18</v>
       </c>
@@ -1635,7 +1641,7 @@
       </c>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A10" s="14"/>
+      <c r="A10" s="30"/>
       <c r="B10" s="3" t="s">
         <v>20</v>
       </c>
@@ -1704,7 +1710,7 @@
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A11" s="14"/>
+      <c r="A11" s="30"/>
       <c r="B11" s="3" t="s">
         <v>22</v>
       </c>
@@ -1773,7 +1779,7 @@
       </c>
     </row>
     <row r="12" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="15"/>
+      <c r="A12" s="31"/>
       <c r="B12" s="4" t="s">
         <v>24</v>
       </c>
@@ -1842,7 +1848,7 @@
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="32" t="s">
         <v>26</v>
       </c>
       <c r="B13" s="3" t="s">
@@ -1913,7 +1919,7 @@
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A14" s="14"/>
+      <c r="A14" s="30"/>
       <c r="B14" s="3" t="s">
         <v>29</v>
       </c>
@@ -1982,7 +1988,7 @@
       </c>
     </row>
     <row r="15" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="15"/>
+      <c r="A15" s="31"/>
       <c r="B15" s="4" t="s">
         <v>31</v>
       </c>
@@ -2122,7 +2128,7 @@
       </c>
     </row>
     <row r="17" spans="1:23" ht="54" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="29" t="s">
         <v>36</v>
       </c>
       <c r="B17" s="3" t="s">
@@ -2193,7 +2199,7 @@
       </c>
     </row>
     <row r="18" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="15"/>
+      <c r="A18" s="31"/>
       <c r="B18" s="4" t="s">
         <v>39</v>
       </c>
@@ -2262,7 +2268,7 @@
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A19" s="16" t="s">
+      <c r="A19" s="32" t="s">
         <v>41</v>
       </c>
       <c r="B19" s="3" t="s">
@@ -2333,7 +2339,7 @@
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A20" s="14"/>
+      <c r="A20" s="30"/>
       <c r="B20" s="3" t="s">
         <v>44</v>
       </c>
@@ -2402,7 +2408,7 @@
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A21" s="14"/>
+      <c r="A21" s="30"/>
       <c r="B21" s="3" t="s">
         <v>46</v>
       </c>
@@ -2471,7 +2477,7 @@
       </c>
     </row>
     <row r="22" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="15"/>
+      <c r="A22" s="31"/>
       <c r="B22" s="4" t="s">
         <v>48</v>
       </c>
@@ -2611,7 +2617,7 @@
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="29" t="s">
         <v>53</v>
       </c>
       <c r="B24" s="3" t="s">
@@ -2682,7 +2688,7 @@
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A25" s="14"/>
+      <c r="A25" s="30"/>
       <c r="B25" s="3" t="s">
         <v>56</v>
       </c>
@@ -2751,7 +2757,7 @@
       </c>
     </row>
     <row r="26" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="15"/>
+      <c r="A26" s="31"/>
       <c r="B26" s="4" t="s">
         <v>58</v>
       </c>
@@ -2891,7 +2897,7 @@
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A28" s="13" t="s">
+      <c r="A28" s="29" t="s">
         <v>63</v>
       </c>
       <c r="B28" s="3" t="s">
@@ -2962,7 +2968,7 @@
       </c>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A29" s="14"/>
+      <c r="A29" s="30"/>
       <c r="B29" s="3" t="s">
         <v>66</v>
       </c>
@@ -3031,7 +3037,7 @@
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A30" s="14"/>
+      <c r="A30" s="30"/>
       <c r="B30" s="3" t="s">
         <v>68</v>
       </c>
@@ -3100,7 +3106,7 @@
       </c>
     </row>
     <row r="31" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="15"/>
+      <c r="A31" s="31"/>
       <c r="B31" s="4" t="s">
         <v>70</v>
       </c>
@@ -3596,11 +3602,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="R1:S1"/>
-    <mergeCell ref="T1:U1"/>
-    <mergeCell ref="V1:W1"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="A7:A12"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="A28:A31"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="F1:G1"/>
@@ -3608,11 +3614,11 @@
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="A19:A22"/>
     <mergeCell ref="A24:A26"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="A7:A12"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="P1:Q1"/>
+    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="T1:U1"/>
+    <mergeCell ref="V1:W1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3621,133 +3627,93 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6803A2EC-9C5B-4557-ACE7-8781747B7323}">
-  <dimension ref="A1:W37"/>
+  <dimension ref="A1:O37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.44140625" customWidth="1"/>
-    <col min="2" max="2" width="17.109375" customWidth="1"/>
+    <col min="1" max="1" width="18.77734375" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="9.77734375" customWidth="1"/>
-    <col min="4" max="23" width="9" customWidth="1"/>
+    <col min="4" max="15" width="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+    <row r="1" spans="1:15" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40" t="s">
+      <c r="B1" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="D1" s="39" t="s">
         <v>90</v>
       </c>
-      <c r="E1" s="28"/>
-      <c r="F1" s="21" t="s">
+      <c r="E1" s="40"/>
+      <c r="F1" s="35" t="s">
         <v>91</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="21" t="s">
+      <c r="G1" s="36"/>
+      <c r="H1" s="35" t="s">
         <v>92</v>
       </c>
-      <c r="I1" s="36"/>
-      <c r="J1" s="21" t="s">
+      <c r="I1" s="41"/>
+      <c r="J1" s="35" t="s">
         <v>93</v>
       </c>
-      <c r="K1" s="22"/>
-      <c r="L1" s="36" t="s">
-        <v>94</v>
-      </c>
-      <c r="M1" s="22"/>
-      <c r="N1" s="21" t="s">
-        <v>95</v>
-      </c>
-      <c r="O1" s="22"/>
-      <c r="P1" s="21" t="s">
-        <v>96</v>
-      </c>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="S1" s="22"/>
-      <c r="T1" s="21" t="s">
-        <v>98</v>
-      </c>
-      <c r="U1" s="22"/>
-      <c r="V1" s="21" t="s">
-        <v>99</v>
-      </c>
-      <c r="W1" s="22"/>
-    </row>
-    <row r="2" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
-      <c r="B2" s="41"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="26" t="s">
+      <c r="K1" s="36"/>
+      <c r="L1" s="41" t="s">
+        <v>108</v>
+      </c>
+      <c r="M1" s="36"/>
+      <c r="N1" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="O1" s="36"/>
+    </row>
+    <row r="2" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="34"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="E2" s="39" t="s">
+      <c r="E2" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="F2" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="G2" s="25" t="s">
+      <c r="G2" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="H2" s="24" t="s">
+      <c r="H2" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="I2" s="24" t="s">
+      <c r="I2" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="J2" s="23" t="s">
+      <c r="J2" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="K2" s="25" t="s">
+      <c r="K2" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="L2" s="24" t="s">
+      <c r="L2" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="M2" s="25" t="s">
+      <c r="M2" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="N2" s="24" t="s">
+      <c r="N2" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="O2" s="25" t="s">
+      <c r="O2" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="P2" s="24" t="s">
-        <v>100</v>
-      </c>
-      <c r="Q2" s="25" t="s">
-        <v>101</v>
-      </c>
-      <c r="R2" s="24" t="s">
-        <v>105</v>
-      </c>
-      <c r="S2" s="25" t="s">
-        <v>106</v>
-      </c>
-      <c r="T2" s="24" t="s">
-        <v>100</v>
-      </c>
-      <c r="U2" s="25" t="s">
-        <v>101</v>
-      </c>
-      <c r="V2" s="24" t="s">
-        <v>105</v>
-      </c>
-      <c r="W2" s="25" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A3" s="29" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
@@ -3756,206 +3722,134 @@
       <c r="C3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="29">
+      <c r="D3" s="16">
         <v>8</v>
       </c>
-      <c r="E3" s="30">
+      <c r="E3" s="17">
         <v>16</v>
       </c>
-      <c r="F3" s="29">
+      <c r="F3" s="16">
         <v>18</v>
       </c>
-      <c r="G3" s="30">
+      <c r="G3" s="17">
         <v>15</v>
       </c>
-      <c r="H3" s="29" t="s">
-        <v>107</v>
-      </c>
-      <c r="I3" s="37" t="s">
-        <v>107</v>
-      </c>
-      <c r="J3" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K3" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L3" s="29">
+      <c r="H3" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="I3" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="J3" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K3" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L3" s="16">
         <v>8</v>
       </c>
-      <c r="M3" s="30">
+      <c r="M3" s="17">
         <v>8</v>
       </c>
-      <c r="N3" s="37">
+      <c r="N3" s="23">
         <v>18</v>
       </c>
-      <c r="O3" s="30">
+      <c r="O3" s="17">
         <v>18</v>
       </c>
-      <c r="P3" s="37" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q3" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="R3" s="29" t="s">
-        <v>107</v>
-      </c>
-      <c r="S3" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="T3" s="29" t="s">
-        <v>107</v>
-      </c>
-      <c r="U3" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="V3" s="37" t="s">
-        <v>107</v>
-      </c>
-      <c r="W3" s="30" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A4" s="14"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A4" s="30"/>
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="31">
+      <c r="D4" s="18">
         <v>2</v>
       </c>
-      <c r="E4" s="32">
+      <c r="E4" s="19">
         <v>4</v>
       </c>
-      <c r="F4" s="31">
+      <c r="F4" s="18">
         <v>17</v>
       </c>
-      <c r="G4" s="32">
+      <c r="G4" s="19">
         <v>14</v>
       </c>
-      <c r="H4" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I4" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J4" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K4" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L4" s="31">
+      <c r="H4" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I4" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J4" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K4" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L4" s="18">
         <v>2</v>
       </c>
-      <c r="M4" s="32">
+      <c r="M4" s="19">
         <v>2</v>
       </c>
-      <c r="N4" s="31">
+      <c r="N4" s="18">
         <v>17</v>
       </c>
-      <c r="O4" s="32">
+      <c r="O4" s="19">
         <v>17</v>
       </c>
-      <c r="P4" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q4" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R4" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S4" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T4" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U4" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V4" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W4" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="15"/>
+    </row>
+    <row r="5" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="31"/>
       <c r="B5" s="4" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="31">
+      <c r="D5" s="18">
         <v>2</v>
       </c>
-      <c r="E5" s="32">
+      <c r="E5" s="19">
         <v>4</v>
       </c>
-      <c r="F5" s="31">
+      <c r="F5" s="18">
         <v>17</v>
       </c>
-      <c r="G5" s="32">
+      <c r="G5" s="19">
         <v>14</v>
       </c>
-      <c r="H5" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I5" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J5" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K5" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L5" s="31">
+      <c r="H5" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J5" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K5" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L5" s="18">
         <v>2</v>
       </c>
-      <c r="M5" s="32">
+      <c r="M5" s="19">
         <v>2</v>
       </c>
-      <c r="N5" s="31">
+      <c r="N5" s="18">
         <v>16</v>
       </c>
-      <c r="O5" s="32">
+      <c r="O5" s="19">
         <v>16</v>
       </c>
-      <c r="P5" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q5" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R5" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S5" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T5" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U5" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V5" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W5" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>10</v>
       </c>
@@ -3965,69 +3859,45 @@
       <c r="C6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="31">
+      <c r="D6" s="18">
         <v>32</v>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="19">
         <v>32</v>
       </c>
-      <c r="F6" s="31">
+      <c r="F6" s="18">
         <v>24</v>
       </c>
-      <c r="G6" s="32">
+      <c r="G6" s="19">
         <v>24</v>
       </c>
-      <c r="H6" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I6" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J6" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K6" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L6" s="31">
+      <c r="H6" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J6" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K6" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L6" s="18">
         <v>32</v>
       </c>
-      <c r="M6" s="32">
+      <c r="M6" s="19">
         <v>32</v>
       </c>
-      <c r="N6" s="31">
+      <c r="N6" s="18">
         <v>21</v>
       </c>
-      <c r="O6" s="32">
+      <c r="O6" s="19">
         <v>21</v>
       </c>
-      <c r="P6" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q6" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R6" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S6" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T6" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U6" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V6" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W6" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7" s="29" t="s">
         <v>13</v>
       </c>
       <c r="B7" s="3" t="s">
@@ -4036,414 +3906,270 @@
       <c r="C7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="31">
+      <c r="D7" s="18">
         <v>8</v>
       </c>
-      <c r="E7" s="32">
+      <c r="E7" s="19">
         <v>8</v>
       </c>
-      <c r="F7" s="31">
+      <c r="F7" s="18">
         <v>14</v>
       </c>
-      <c r="G7" s="32">
+      <c r="G7" s="19">
         <v>14</v>
       </c>
-      <c r="H7" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I7" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J7" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K7" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L7" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M7" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N7" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O7" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P7" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q7" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R7" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S7" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T7" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U7" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V7" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W7" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A8" s="14"/>
+      <c r="H7" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J7" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K7" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L7" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M7" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N7" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O7" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A8" s="30"/>
       <c r="B8" s="3" t="s">
         <v>16</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="31">
+      <c r="D8" s="18">
         <v>8</v>
       </c>
-      <c r="E8" s="32">
+      <c r="E8" s="19">
         <v>8</v>
       </c>
-      <c r="F8" s="31" t="s">
+      <c r="F8" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="G8" s="32" t="s">
+      <c r="G8" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="H8" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I8" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J8" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K8" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L8" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M8" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N8" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O8" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P8" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q8" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R8" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S8" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T8" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U8" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V8" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W8" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A9" s="14"/>
+      <c r="H8" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J8" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K8" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L8" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M8" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N8" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O8" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A9" s="30"/>
       <c r="B9" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="31">
+      <c r="D9" s="18">
         <v>8</v>
       </c>
-      <c r="E9" s="32">
+      <c r="E9" s="19">
         <v>8</v>
       </c>
-      <c r="F9" s="31">
+      <c r="F9" s="18">
         <v>15</v>
       </c>
-      <c r="G9" s="32">
+      <c r="G9" s="19">
         <v>15</v>
       </c>
-      <c r="H9" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I9" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J9" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K9" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L9" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M9" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N9" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O9" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P9" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q9" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R9" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S9" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T9" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U9" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V9" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W9" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A10" s="14"/>
+      <c r="H9" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J9" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K9" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L9" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M9" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N9" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O9" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A10" s="30"/>
       <c r="B10" s="3" t="s">
         <v>20</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="31" t="s">
+      <c r="D10" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="E10" s="32" t="s">
+      <c r="E10" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="F10" s="31" t="s">
+      <c r="F10" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="G10" s="32" t="s">
+      <c r="G10" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="H10" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I10" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J10" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K10" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L10" s="31">
+      <c r="H10" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I10" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J10" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K10" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L10" s="18">
         <v>1E-3</v>
       </c>
-      <c r="M10" s="32">
+      <c r="M10" s="19">
         <v>16</v>
       </c>
-      <c r="N10" s="31">
+      <c r="N10" s="18">
         <v>50</v>
       </c>
-      <c r="O10" s="32">
+      <c r="O10" s="19">
         <v>17</v>
       </c>
-      <c r="P10" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q10" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R10" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S10" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T10" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U10" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V10" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W10" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A11" s="14"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A11" s="30"/>
       <c r="B11" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="31">
+      <c r="D11" s="18">
         <v>8</v>
       </c>
-      <c r="E11" s="32">
+      <c r="E11" s="19">
         <v>16</v>
       </c>
-      <c r="F11" s="31">
+      <c r="F11" s="18">
         <v>23</v>
       </c>
-      <c r="G11" s="32">
+      <c r="G11" s="19">
         <v>20</v>
       </c>
-      <c r="H11" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I11" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J11" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K11" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L11" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M11" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N11" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O11" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P11" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q11" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R11" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S11" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T11" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U11" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V11" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W11" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="15"/>
+      <c r="H11" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I11" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J11" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K11" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L11" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M11" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N11" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O11" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="31"/>
       <c r="B12" s="4" t="s">
         <v>24</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="31">
+      <c r="D12" s="18">
         <v>8</v>
       </c>
-      <c r="E12" s="32">
+      <c r="E12" s="19">
         <v>16</v>
       </c>
-      <c r="F12" s="31">
+      <c r="F12" s="18">
         <v>20</v>
       </c>
-      <c r="G12" s="32">
+      <c r="G12" s="19">
         <v>17</v>
       </c>
-      <c r="H12" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I12" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J12" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K12" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L12" s="31">
+      <c r="H12" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J12" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K12" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L12" s="18">
         <v>8</v>
       </c>
-      <c r="M12" s="32">
+      <c r="M12" s="19">
         <v>8</v>
       </c>
-      <c r="N12" s="31">
+      <c r="N12" s="18">
         <v>20</v>
       </c>
-      <c r="O12" s="32">
+      <c r="O12" s="19">
         <v>20</v>
       </c>
-      <c r="P12" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q12" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R12" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S12" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T12" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U12" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V12" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W12" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="13" spans="1:23" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="16" t="s">
+    </row>
+    <row r="13" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="32" t="s">
         <v>26</v>
       </c>
       <c r="B13" s="3" t="s">
@@ -4452,206 +4178,134 @@
       <c r="C13" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="31">
+      <c r="D13" s="18">
         <v>8</v>
       </c>
-      <c r="E13" s="32">
+      <c r="E13" s="19">
         <v>8</v>
       </c>
-      <c r="F13" s="31">
+      <c r="F13" s="18">
         <v>19</v>
       </c>
-      <c r="G13" s="32">
+      <c r="G13" s="19">
         <v>19</v>
       </c>
-      <c r="H13" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I13" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J13" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K13" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L13" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M13" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N13" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O13" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P13" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q13" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R13" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S13" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T13" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U13" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V13" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W13" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="14" spans="1:23" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="14"/>
+      <c r="H13" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I13" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J13" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K13" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L13" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M13" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N13" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O13" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="30"/>
       <c r="B14" s="3" t="s">
         <v>29</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="31">
+      <c r="D14" s="18">
         <v>8</v>
       </c>
-      <c r="E14" s="32">
+      <c r="E14" s="19">
         <v>16</v>
       </c>
-      <c r="F14" s="31">
+      <c r="F14" s="18">
         <v>20</v>
       </c>
-      <c r="G14" s="32">
+      <c r="G14" s="19">
         <v>17</v>
       </c>
-      <c r="H14" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I14" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J14" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K14" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L14" s="31">
+      <c r="H14" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J14" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K14" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L14" s="18">
         <v>8</v>
       </c>
-      <c r="M14" s="32">
+      <c r="M14" s="19">
         <v>8</v>
       </c>
-      <c r="N14" s="31">
+      <c r="N14" s="18">
         <v>20</v>
       </c>
-      <c r="O14" s="32">
+      <c r="O14" s="19">
         <v>20</v>
       </c>
-      <c r="P14" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q14" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R14" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S14" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T14" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U14" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V14" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W14" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="15" spans="1:23" ht="42" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="15"/>
+    </row>
+    <row r="15" spans="1:15" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="31"/>
       <c r="B15" s="4" t="s">
         <v>31</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="31">
+      <c r="D15" s="18">
         <v>8</v>
       </c>
-      <c r="E15" s="32">
+      <c r="E15" s="19">
         <v>16</v>
       </c>
-      <c r="F15" s="31">
+      <c r="F15" s="18">
         <v>23</v>
       </c>
-      <c r="G15" s="32">
+      <c r="G15" s="19">
         <v>20</v>
       </c>
-      <c r="H15" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I15" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J15" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K15" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L15" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M15" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N15" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O15" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P15" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q15" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R15" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S15" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T15" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U15" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V15" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W15" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="H15" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J15" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K15" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L15" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M15" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N15" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O15" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
         <v>33</v>
       </c>
@@ -4661,69 +4315,45 @@
       <c r="C16" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D16" s="31">
+      <c r="D16" s="18">
         <v>16</v>
       </c>
-      <c r="E16" s="32">
+      <c r="E16" s="19">
         <v>16</v>
       </c>
-      <c r="F16" s="31">
+      <c r="F16" s="18">
         <v>14</v>
       </c>
-      <c r="G16" s="32">
+      <c r="G16" s="19">
         <v>14</v>
       </c>
-      <c r="H16" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I16" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J16" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K16" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L16" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M16" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N16" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O16" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P16" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q16" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R16" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S16" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T16" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U16" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V16" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W16" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A17" s="13" t="s">
+      <c r="H16" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I16" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J16" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K16" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L16" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M16" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N16" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O16" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A17" s="29" t="s">
         <v>36</v>
       </c>
       <c r="B17" s="3" t="s">
@@ -4732,138 +4362,90 @@
       <c r="C17" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D17" s="31">
+      <c r="D17" s="18">
         <v>8</v>
       </c>
-      <c r="E17" s="32">
+      <c r="E17" s="19">
         <v>8</v>
       </c>
-      <c r="F17" s="31">
+      <c r="F17" s="18">
         <v>19</v>
       </c>
-      <c r="G17" s="32">
+      <c r="G17" s="19">
         <v>19</v>
       </c>
-      <c r="H17" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I17" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J17" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K17" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L17" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M17" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N17" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O17" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P17" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q17" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R17" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S17" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T17" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U17" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V17" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W17" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="18" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="15"/>
+      <c r="H17" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I17" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J17" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K17" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L17" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M17" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N17" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O17" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="31"/>
       <c r="B18" s="4" t="s">
         <v>39</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D18" s="31" t="s">
+      <c r="D18" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="E18" s="32" t="s">
+      <c r="E18" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="F18" s="31">
+      <c r="F18" s="18">
         <v>19</v>
       </c>
-      <c r="G18" s="32">
+      <c r="G18" s="19">
         <v>19</v>
       </c>
-      <c r="H18" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I18" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J18" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K18" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L18" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M18" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N18" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O18" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P18" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q18" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R18" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S18" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T18" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U18" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V18" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W18" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A19" s="16" t="s">
+      <c r="H18" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I18" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J18" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K18" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L18" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M18" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N18" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O18" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A19" s="32" t="s">
         <v>41</v>
       </c>
       <c r="B19" s="3" t="s">
@@ -4872,275 +4454,179 @@
       <c r="C19" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D19" s="31">
+      <c r="D19" s="18">
         <v>1</v>
       </c>
-      <c r="E19" s="32">
+      <c r="E19" s="19">
         <v>4</v>
       </c>
-      <c r="F19" s="31">
+      <c r="F19" s="18">
         <v>22</v>
       </c>
-      <c r="G19" s="32">
+      <c r="G19" s="19">
         <v>19</v>
       </c>
-      <c r="H19" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I19" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J19" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K19" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L19" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M19" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N19" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O19" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P19" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q19" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R19" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S19" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T19" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U19" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V19" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W19" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A20" s="14"/>
+      <c r="H19" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I19" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J19" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K19" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L19" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M19" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N19" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O19" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A20" s="30"/>
       <c r="B20" s="3" t="s">
         <v>44</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D20" s="31">
+      <c r="D20" s="18">
         <v>1</v>
       </c>
-      <c r="E20" s="32">
+      <c r="E20" s="19">
         <v>1</v>
       </c>
-      <c r="F20" s="31">
+      <c r="F20" s="18">
         <v>17</v>
       </c>
-      <c r="G20" s="32">
+      <c r="G20" s="19">
         <v>17</v>
       </c>
-      <c r="H20" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I20" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J20" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K20" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L20" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M20" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N20" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O20" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P20" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q20" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R20" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S20" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T20" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U20" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V20" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W20" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A21" s="14"/>
+      <c r="H20" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I20" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J20" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K20" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L20" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M20" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N20" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O20" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A21" s="30"/>
       <c r="B21" s="3" t="s">
         <v>46</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="31">
+      <c r="D21" s="18">
         <v>1</v>
       </c>
-      <c r="E21" s="32">
+      <c r="E21" s="19">
         <v>2</v>
       </c>
-      <c r="F21" s="31">
+      <c r="F21" s="18">
         <v>25</v>
       </c>
-      <c r="G21" s="32">
+      <c r="G21" s="19">
         <v>22</v>
       </c>
-      <c r="H21" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I21" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J21" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K21" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L21" s="31">
+      <c r="H21" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I21" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J21" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K21" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L21" s="18">
         <v>1</v>
       </c>
-      <c r="M21" s="32">
+      <c r="M21" s="19">
         <v>1</v>
       </c>
-      <c r="N21" s="31">
+      <c r="N21" s="18">
         <v>25</v>
       </c>
-      <c r="O21" s="32">
+      <c r="O21" s="19">
         <v>25</v>
       </c>
-      <c r="P21" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q21" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R21" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S21" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T21" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U21" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V21" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W21" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="22" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="15"/>
+    </row>
+    <row r="22" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="31"/>
       <c r="B22" s="4" t="s">
         <v>48</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="D22" s="31">
+      <c r="D22" s="18">
         <v>1</v>
       </c>
-      <c r="E22" s="32">
+      <c r="E22" s="19">
         <v>2</v>
       </c>
-      <c r="F22" s="31">
+      <c r="F22" s="18">
         <v>20</v>
       </c>
-      <c r="G22" s="32">
+      <c r="G22" s="19">
         <v>17</v>
       </c>
-      <c r="H22" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I22" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J22" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K22" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L22" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M22" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N22" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O22" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P22" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q22" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R22" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S22" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T22" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U22" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V22" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W22" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="23" spans="1:23" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="H22" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I22" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J22" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K22" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L22" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M22" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N22" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O22" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="s">
         <v>50</v>
       </c>
@@ -5150,69 +4636,45 @@
       <c r="C23" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D23" s="31">
+      <c r="D23" s="18">
         <v>1</v>
       </c>
-      <c r="E23" s="32">
+      <c r="E23" s="19">
         <v>4</v>
       </c>
-      <c r="F23" s="31">
+      <c r="F23" s="18">
         <v>27</v>
       </c>
-      <c r="G23" s="32">
+      <c r="G23" s="19">
         <v>24</v>
       </c>
-      <c r="H23" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I23" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J23" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K23" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L23" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M23" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N23" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O23" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P23" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q23" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R23" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S23" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T23" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U23" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V23" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W23" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A24" s="13" t="s">
+      <c r="H23" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I23" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J23" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K23" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L23" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M23" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N23" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O23" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A24" s="29" t="s">
         <v>53</v>
       </c>
       <c r="B24" s="3" t="s">
@@ -5221,206 +4683,134 @@
       <c r="C24" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D24" s="31">
+      <c r="D24" s="18">
         <v>0.5</v>
       </c>
-      <c r="E24" s="32">
+      <c r="E24" s="19">
         <v>1</v>
       </c>
-      <c r="F24" s="31">
+      <c r="F24" s="18">
         <v>25</v>
       </c>
-      <c r="G24" s="32">
+      <c r="G24" s="19">
         <v>22</v>
       </c>
-      <c r="H24" s="31">
+      <c r="H24" s="18">
         <v>0.5</v>
       </c>
-      <c r="I24" s="20">
+      <c r="I24" s="11">
         <v>0.5</v>
       </c>
-      <c r="J24" s="31">
+      <c r="J24" s="18">
         <v>25</v>
       </c>
-      <c r="K24" s="32">
+      <c r="K24" s="19">
         <v>25</v>
       </c>
-      <c r="L24" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M24" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N24" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O24" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P24" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q24" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R24" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S24" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T24" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U24" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V24" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W24" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A25" s="14"/>
+      <c r="L24" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M24" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N24" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O24" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A25" s="30"/>
       <c r="B25" s="3" t="s">
         <v>56</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D25" s="31">
+      <c r="D25" s="18">
         <v>2</v>
       </c>
-      <c r="E25" s="32">
+      <c r="E25" s="19">
         <v>8</v>
       </c>
-      <c r="F25" s="31">
+      <c r="F25" s="18">
         <v>22</v>
       </c>
-      <c r="G25" s="32">
+      <c r="G25" s="19">
         <v>16</v>
       </c>
-      <c r="H25" s="31">
+      <c r="H25" s="18">
         <v>2</v>
       </c>
-      <c r="I25" s="20">
+      <c r="I25" s="11">
         <v>4</v>
       </c>
-      <c r="J25" s="31">
+      <c r="J25" s="18">
         <v>22</v>
       </c>
-      <c r="K25" s="32">
+      <c r="K25" s="19">
         <v>17</v>
       </c>
-      <c r="L25" s="31">
+      <c r="L25" s="18">
         <v>2</v>
       </c>
-      <c r="M25" s="32">
+      <c r="M25" s="19">
         <v>4</v>
       </c>
-      <c r="N25" s="31">
+      <c r="N25" s="18">
         <v>22</v>
       </c>
-      <c r="O25" s="32">
+      <c r="O25" s="19">
         <v>19</v>
       </c>
-      <c r="P25" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q25" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R25" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S25" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T25" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U25" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V25" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W25" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="26" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="15"/>
+    </row>
+    <row r="26" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="31"/>
       <c r="B26" s="4" t="s">
         <v>58</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D26" s="31">
+      <c r="D26" s="18">
         <v>2</v>
       </c>
-      <c r="E26" s="32">
+      <c r="E26" s="19">
         <v>8</v>
       </c>
-      <c r="F26" s="31">
+      <c r="F26" s="18">
         <v>22</v>
       </c>
-      <c r="G26" s="32">
+      <c r="G26" s="19">
         <v>16</v>
       </c>
-      <c r="H26" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I26" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J26" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K26" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L26" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M26" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N26" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O26" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P26" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q26" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R26" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S26" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T26" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U26" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V26" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W26" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="27" spans="1:23" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="H26" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I26" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J26" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K26" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L26" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M26" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N26" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O26" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" ht="33.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
         <v>60</v>
       </c>
@@ -5430,69 +4820,45 @@
       <c r="C27" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D27" s="31">
+      <c r="D27" s="18">
         <v>64</v>
       </c>
-      <c r="E27" s="32">
+      <c r="E27" s="19">
         <v>64</v>
       </c>
-      <c r="F27" s="31">
+      <c r="F27" s="18">
         <v>11</v>
       </c>
-      <c r="G27" s="32">
+      <c r="G27" s="19">
         <v>11</v>
       </c>
-      <c r="H27" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I27" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J27" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K27" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L27" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M27" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N27" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O27" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P27" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q27" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R27" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S27" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T27" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U27" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V27" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W27" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="28" spans="1:23" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="13" t="s">
+      <c r="H27" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I27" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J27" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K27" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L27" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M27" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N27" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O27" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A28" s="29" t="s">
         <v>63</v>
       </c>
       <c r="B28" s="3" t="s">
@@ -5501,275 +4867,179 @@
       <c r="C28" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D28" s="31">
+      <c r="D28" s="18">
         <v>0.25</v>
       </c>
-      <c r="E28" s="32">
+      <c r="E28" s="19">
         <v>0.5</v>
       </c>
-      <c r="F28" s="31">
+      <c r="F28" s="18">
         <v>26</v>
       </c>
-      <c r="G28" s="32">
+      <c r="G28" s="19">
         <v>24</v>
       </c>
-      <c r="H28" s="31">
+      <c r="H28" s="18">
         <v>0.25</v>
       </c>
-      <c r="I28" s="20">
+      <c r="I28" s="11">
         <v>0.5</v>
       </c>
-      <c r="J28" s="31">
+      <c r="J28" s="18">
         <v>25</v>
       </c>
-      <c r="K28" s="32">
+      <c r="K28" s="19">
         <v>22</v>
       </c>
-      <c r="L28" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M28" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N28" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O28" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P28" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q28" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R28" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S28" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T28" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U28" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V28" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W28" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="29" spans="1:23" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="14"/>
+      <c r="L28" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M28" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N28" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O28" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A29" s="30"/>
       <c r="B29" s="3" t="s">
         <v>66</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D29" s="31">
+      <c r="D29" s="18">
         <v>0.5</v>
       </c>
-      <c r="E29" s="32">
+      <c r="E29" s="19">
         <v>1</v>
       </c>
-      <c r="F29" s="31">
+      <c r="F29" s="18">
         <v>23</v>
       </c>
-      <c r="G29" s="32">
+      <c r="G29" s="19">
         <v>19</v>
       </c>
-      <c r="H29" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I29" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J29" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K29" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L29" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M29" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N29" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O29" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P29" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q29" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R29" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S29" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T29" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U29" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V29" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W29" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A30" s="14"/>
+      <c r="H29" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I29" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J29" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K29" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L29" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M29" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N29" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O29" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A30" s="30"/>
       <c r="B30" s="3" t="s">
         <v>68</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="D30" s="31">
+      <c r="D30" s="18">
         <v>0.5</v>
       </c>
-      <c r="E30" s="32">
+      <c r="E30" s="19">
         <v>1</v>
       </c>
-      <c r="F30" s="31">
+      <c r="F30" s="18">
         <v>22</v>
       </c>
-      <c r="G30" s="32">
+      <c r="G30" s="19">
         <v>19</v>
       </c>
-      <c r="H30" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I30" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J30" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K30" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L30" s="31">
+      <c r="H30" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I30" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J30" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K30" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L30" s="18">
         <v>0.5</v>
       </c>
-      <c r="M30" s="32">
+      <c r="M30" s="19">
         <v>0.5</v>
       </c>
-      <c r="N30" s="31">
+      <c r="N30" s="18">
         <v>22</v>
       </c>
-      <c r="O30" s="32">
+      <c r="O30" s="19">
         <v>22</v>
       </c>
-      <c r="P30" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q30" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R30" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S30" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T30" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U30" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V30" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W30" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="31" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="15"/>
+    </row>
+    <row r="31" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="31"/>
       <c r="B31" s="4" t="s">
         <v>70</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D31" s="31">
+      <c r="D31" s="18">
         <v>0.25</v>
       </c>
-      <c r="E31" s="32">
+      <c r="E31" s="19">
         <v>0.5</v>
       </c>
-      <c r="F31" s="31">
+      <c r="F31" s="18">
         <v>24</v>
       </c>
-      <c r="G31" s="32">
+      <c r="G31" s="19">
         <v>22</v>
       </c>
-      <c r="H31" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I31" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J31" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K31" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L31" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M31" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N31" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O31" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P31" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q31" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R31" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S31" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T31" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U31" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V31" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W31" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="32" spans="1:23" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="H31" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I31" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J31" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K31" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L31" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M31" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N31" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O31" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
         <v>72</v>
       </c>
@@ -5779,68 +5049,44 @@
       <c r="C32" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="D32" s="33" t="s">
+      <c r="D32" s="20" t="s">
         <v>103</v>
       </c>
       <c r="E32" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="F32" s="33" t="s">
+      <c r="F32" s="20" t="s">
         <v>103</v>
       </c>
       <c r="G32" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="H32" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I32" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J32" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K32" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L32" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M32" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N32" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O32" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P32" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q32" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R32" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S32" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T32" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U32" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V32" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W32" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="33" spans="1:23" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="H32" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I32" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J32" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K32" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L32" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M32" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N32" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O32" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
         <v>75</v>
       </c>
@@ -5850,68 +5096,44 @@
       <c r="C33" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="D33" s="31">
+      <c r="D33" s="18">
         <v>2</v>
       </c>
-      <c r="E33" s="32">
+      <c r="E33" s="19">
         <v>4</v>
       </c>
-      <c r="F33" s="31">
+      <c r="F33" s="18">
         <v>14</v>
       </c>
-      <c r="G33" s="32">
+      <c r="G33" s="19">
         <v>11</v>
       </c>
-      <c r="H33" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I33" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J33" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K33" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L33" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M33" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N33" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O33" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P33" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q33" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R33" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S33" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T33" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U33" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V33" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W33" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="34" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="H33" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I33" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J33" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K33" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L33" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M33" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N33" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O33" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
         <v>78</v>
       </c>
@@ -5921,68 +5143,44 @@
       <c r="C34" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="D34" s="31">
+      <c r="D34" s="18">
         <v>1</v>
       </c>
-      <c r="E34" s="32">
+      <c r="E34" s="19">
         <v>4</v>
       </c>
-      <c r="F34" s="31">
+      <c r="F34" s="18">
         <v>26</v>
       </c>
-      <c r="G34" s="32">
+      <c r="G34" s="19">
         <v>21</v>
       </c>
-      <c r="H34" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I34" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J34" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K34" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L34" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M34" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N34" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O34" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P34" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q34" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R34" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S34" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T34" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U34" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V34" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W34" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="35" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="H34" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I34" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J34" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K34" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L34" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M34" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N34" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O34" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>81</v>
       </c>
@@ -5992,68 +5190,44 @@
       <c r="C35" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="D35" s="31">
+      <c r="D35" s="18">
         <v>2</v>
       </c>
-      <c r="E35" s="32">
+      <c r="E35" s="19">
         <v>2</v>
       </c>
-      <c r="F35" s="33" t="s">
+      <c r="F35" s="20" t="s">
         <v>102</v>
       </c>
       <c r="G35" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="H35" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="I35" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J35" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="K35" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L35" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M35" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N35" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O35" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P35" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q35" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R35" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S35" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T35" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U35" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V35" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W35" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="36" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="H35" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I35" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="J35" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K35" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L35" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M35" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N35" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O35" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
         <v>84</v>
       </c>
@@ -6063,68 +5237,44 @@
       <c r="C36" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D36" s="31">
+      <c r="D36" s="18">
         <v>1</v>
       </c>
-      <c r="E36" s="32">
+      <c r="E36" s="19">
         <v>2</v>
       </c>
-      <c r="F36" s="31">
+      <c r="F36" s="18">
         <v>18</v>
       </c>
-      <c r="G36" s="32">
+      <c r="G36" s="19">
         <v>15</v>
       </c>
-      <c r="H36" s="31">
+      <c r="H36" s="18">
         <v>0.5</v>
       </c>
-      <c r="I36" s="20">
+      <c r="I36" s="11">
         <v>0.5</v>
       </c>
-      <c r="J36" s="31">
+      <c r="J36" s="18">
         <v>18</v>
       </c>
-      <c r="K36" s="32">
+      <c r="K36" s="19">
         <v>18</v>
       </c>
-      <c r="L36" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="M36" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="N36" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O36" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="P36" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q36" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="R36" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="S36" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="T36" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="U36" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="V36" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="W36" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="37" spans="1:23" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L36" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M36" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="N36" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="O36" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
         <v>87</v>
       </c>
@@ -6134,89 +5284,61 @@
       <c r="C37" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D37" s="34">
+      <c r="D37" s="21">
         <v>2</v>
       </c>
-      <c r="E37" s="35">
+      <c r="E37" s="22">
         <v>4</v>
       </c>
-      <c r="F37" s="34">
+      <c r="F37" s="21">
         <v>18</v>
       </c>
-      <c r="G37" s="35">
+      <c r="G37" s="22">
         <v>15</v>
       </c>
-      <c r="H37" s="34">
+      <c r="H37" s="21">
         <v>1</v>
       </c>
-      <c r="I37" s="38">
+      <c r="I37" s="24">
         <v>4</v>
       </c>
-      <c r="J37" s="34">
+      <c r="J37" s="21">
         <v>26</v>
       </c>
-      <c r="K37" s="35">
+      <c r="K37" s="22">
         <v>21</v>
       </c>
-      <c r="L37" s="34">
+      <c r="L37" s="21">
         <v>4</v>
       </c>
-      <c r="M37" s="35">
+      <c r="M37" s="22">
         <v>4</v>
       </c>
-      <c r="N37" s="34">
+      <c r="N37" s="21">
         <v>15</v>
       </c>
-      <c r="O37" s="35">
+      <c r="O37" s="22">
         <v>15</v>
       </c>
-      <c r="P37" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q37" s="35" t="s">
-        <v>107</v>
-      </c>
-      <c r="R37" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="S37" s="35" t="s">
-        <v>107</v>
-      </c>
-      <c r="T37" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="U37" s="35" t="s">
-        <v>107</v>
-      </c>
-      <c r="V37" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="W37" s="35" t="s">
-        <v>107</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="16">
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="A7:A12"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="N1:O1"/>
     <mergeCell ref="A13:A15"/>
     <mergeCell ref="A17:A18"/>
     <mergeCell ref="A19:A22"/>
     <mergeCell ref="A24:A26"/>
     <mergeCell ref="A28:A31"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="R1:S1"/>
-    <mergeCell ref="T1:U1"/>
-    <mergeCell ref="V1:W1"/>
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="A7:A12"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="N1:O1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>